<commit_message>
added documentation and fixed hpc shell script
</commit_message>
<xml_diff>
--- a/Results/pam_parametrizer_diagnostics_ecolicore_before.xlsx
+++ b/Results/pam_parametrizer_diagnostics_ecolicore_before.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="35">
   <si>
     <t>run_id</t>
   </si>
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -515,7 +515,7 @@
         <v>19</v>
       </c>
       <c r="E2">
-        <v>1.991839736458246</v>
+        <v>3.831111135630223</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -535,7 +535,7 @@
         <v>20</v>
       </c>
       <c r="E3">
-        <v>14.78965268571219</v>
+        <v>13.6220740898523</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -575,7 +575,7 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>22.6542525417609</v>
+        <v>25.25252525252526</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -595,10 +595,10 @@
         <v>23</v>
       </c>
       <c r="E6">
-        <v>296.2517247666116</v>
+        <v>153.7640148785883</v>
       </c>
       <c r="F6">
-        <v>-0.3516226142591197</v>
+        <v>0.2136029259157772</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -615,10 +615,10 @@
         <v>24</v>
       </c>
       <c r="E7">
-        <v>23723.63770252172</v>
+        <v>2051.565119953358</v>
       </c>
       <c r="F7">
-        <v>-0.3516226142591197</v>
+        <v>0.2136029259157772</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -635,10 +635,10 @@
         <v>19</v>
       </c>
       <c r="E8">
-        <v>112.3408849217983</v>
+        <v>46.67223228368888</v>
       </c>
       <c r="F8">
-        <v>-0.3516226142591197</v>
+        <v>0.2136029259157772</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -655,10 +655,10 @@
         <v>20</v>
       </c>
       <c r="E9">
-        <v>988.8191864745676</v>
+        <v>514.8877794904437</v>
       </c>
       <c r="F9">
-        <v>-0.3516226142591197</v>
+        <v>0.2136029259157772</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -675,10 +675,10 @@
         <v>25</v>
       </c>
       <c r="E10">
-        <v>133.0872555012624</v>
+        <v>75.14405193805221</v>
       </c>
       <c r="F10">
-        <v>0.6426266713201126</v>
+        <v>0.6185069514077962</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -695,10 +695,10 @@
         <v>26</v>
       </c>
       <c r="E11">
-        <v>693.6884172422936</v>
+        <v>46.34339474774187</v>
       </c>
       <c r="F11">
-        <v>0.6426266713201126</v>
+        <v>0.6185069514077962</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -715,10 +715,10 @@
         <v>22</v>
       </c>
       <c r="E12">
-        <v>6020.718804863494</v>
+        <v>173.6843490604816</v>
       </c>
       <c r="F12">
-        <v>0.6426266713201126</v>
+        <v>0.6185069514077962</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -735,10 +735,10 @@
         <v>27</v>
       </c>
       <c r="E13">
-        <v>306.7239748083061</v>
+        <v>83.78751731593059</v>
       </c>
       <c r="F13">
-        <v>0.6426266713201126</v>
+        <v>0.6185069514077962</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -755,10 +755,10 @@
         <v>28</v>
       </c>
       <c r="E14">
-        <v>81.2747963506405</v>
+        <v>527.3919620034662</v>
       </c>
       <c r="F14">
-        <v>0.7335995757615115</v>
+        <v>0.6200091631213471</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -775,10 +775,10 @@
         <v>29</v>
       </c>
       <c r="E15">
-        <v>3.27537326822564</v>
+        <v>2.477454938237429</v>
       </c>
       <c r="F15">
-        <v>0.7335995757615115</v>
+        <v>0.6200091631213471</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -795,10 +795,10 @@
         <v>30</v>
       </c>
       <c r="E16">
-        <v>73.88689394275244</v>
+        <v>22.79964968423831</v>
       </c>
       <c r="F16">
-        <v>0.7335995757615115</v>
+        <v>0.6200091631213471</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -815,10 +815,570 @@
         <v>31</v>
       </c>
       <c r="E17">
-        <v>173.3982338335322</v>
+        <v>64.42402581512842</v>
       </c>
       <c r="F17">
-        <v>0.7335995757615115</v>
+        <v>0.6200091631213471</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18">
+        <v>164.209369743447</v>
+      </c>
+      <c r="F18">
+        <v>0.6186929979819762</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19">
+        <v>2.214804273941737</v>
+      </c>
+      <c r="F19">
+        <v>0.6186929979819762</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20">
+        <v>25.9386309433859</v>
+      </c>
+      <c r="F20">
+        <v>0.6186929979819762</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21">
+        <v>9274.086261728185</v>
+      </c>
+      <c r="F21">
+        <v>0.6186929979819762</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22">
+        <v>229.6727819180724</v>
+      </c>
+      <c r="F22">
+        <v>0.6181514447004339</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23">
+        <v>2.213524763781034</v>
+      </c>
+      <c r="F23">
+        <v>0.6181514447004339</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24">
+        <v>46.3955596190448</v>
+      </c>
+      <c r="F24">
+        <v>0.6181514447004339</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25">
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25">
+        <v>1559.02730814162</v>
+      </c>
+      <c r="F25">
+        <v>0.6181514447004339</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26">
+        <v>6</v>
+      </c>
+      <c r="B26" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26">
+        <v>42.79413410255726</v>
+      </c>
+      <c r="F26">
+        <v>0.6208315410287218</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" t="s">
+        <v>29</v>
+      </c>
+      <c r="E27">
+        <v>2.343943983719563</v>
+      </c>
+      <c r="F27">
+        <v>0.6208315410287218</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28">
+        <v>6</v>
+      </c>
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28">
+        <v>20.07522151563619</v>
+      </c>
+      <c r="F28">
+        <v>0.6208315410287218</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29">
+        <v>6</v>
+      </c>
+      <c r="B29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29">
+        <v>518.0772537420993</v>
+      </c>
+      <c r="F29">
+        <v>0.6208315410287218</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30">
+        <v>120.6640731912083</v>
+      </c>
+      <c r="F30">
+        <v>0.6197968074098716</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31">
+        <v>7</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" t="s">
+        <v>29</v>
+      </c>
+      <c r="E31">
+        <v>2.343943983719563</v>
+      </c>
+      <c r="F31">
+        <v>0.6197968074098716</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32">
+        <v>7</v>
+      </c>
+      <c r="B32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E32">
+        <v>24.76726425798622</v>
+      </c>
+      <c r="F32">
+        <v>0.6197968074098716</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33">
+        <v>7</v>
+      </c>
+      <c r="B33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" t="s">
+        <v>31</v>
+      </c>
+      <c r="E33">
+        <v>124.1853441424257</v>
+      </c>
+      <c r="F33">
+        <v>0.6197968074098716</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34">
+        <v>8</v>
+      </c>
+      <c r="B34" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34">
+        <v>98.19936131466052</v>
+      </c>
+      <c r="F34">
+        <v>0.6190405353458538</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35">
+        <v>8</v>
+      </c>
+      <c r="B35" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" t="s">
+        <v>29</v>
+      </c>
+      <c r="E35">
+        <v>2.343943983719563</v>
+      </c>
+      <c r="F35">
+        <v>0.6190405353458538</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36">
+        <v>8</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" t="s">
+        <v>30</v>
+      </c>
+      <c r="E36">
+        <v>38.682239708945</v>
+      </c>
+      <c r="F36">
+        <v>0.6190405353458538</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37">
+        <v>8</v>
+      </c>
+      <c r="B37" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" t="s">
+        <v>31</v>
+      </c>
+      <c r="E37">
+        <v>124.1853441424257</v>
+      </c>
+      <c r="F37">
+        <v>0.6190405353458538</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" t="s">
+        <v>28</v>
+      </c>
+      <c r="E38">
+        <v>198.5855843670347</v>
+      </c>
+      <c r="F38">
+        <v>0.6222684942896206</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39">
+        <v>9</v>
+      </c>
+      <c r="B39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" t="s">
+        <v>29</v>
+      </c>
+      <c r="E39">
+        <v>2.477454938237429</v>
+      </c>
+      <c r="F39">
+        <v>0.6222684942896206</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40">
+        <v>9</v>
+      </c>
+      <c r="B40" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" t="s">
+        <v>30</v>
+      </c>
+      <c r="E40">
+        <v>11.12092308522421</v>
+      </c>
+      <c r="F40">
+        <v>0.6222684942896206</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41">
+        <v>9</v>
+      </c>
+      <c r="B41" t="s">
+        <v>17</v>
+      </c>
+      <c r="C41" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" t="s">
+        <v>31</v>
+      </c>
+      <c r="E41">
+        <v>96.31262526200777</v>
+      </c>
+      <c r="F41">
+        <v>0.6222684942896206</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42">
+        <v>10</v>
+      </c>
+      <c r="B42" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" t="s">
+        <v>28</v>
+      </c>
+      <c r="E42">
+        <v>28.75904191424239</v>
+      </c>
+      <c r="F42">
+        <v>0.6214922342981547</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43">
+        <v>10</v>
+      </c>
+      <c r="B43" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" t="s">
+        <v>29</v>
+      </c>
+      <c r="E43">
+        <v>2.477454938237429</v>
+      </c>
+      <c r="F43">
+        <v>0.6214922342981547</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" t="s">
+        <v>30</v>
+      </c>
+      <c r="E44">
+        <v>22.43029563008922</v>
+      </c>
+      <c r="F44">
+        <v>0.6214922342981547</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45">
+        <v>10</v>
+      </c>
+      <c r="B45" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" t="s">
+        <v>31</v>
+      </c>
+      <c r="E45">
+        <v>331.5694898768202</v>
+      </c>
+      <c r="F45">
+        <v>0.6214922342981547</v>
       </c>
     </row>
   </sheetData>
@@ -828,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -847,10 +1407,10 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>183.1801338460027</v>
+        <v>180.6590816560201</v>
       </c>
       <c r="C2">
-        <v>0.05088337051277853</v>
+        <v>0.05018307823778337</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -858,10 +1418,10 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>158.9479099659984</v>
+        <v>122.6941453119798</v>
       </c>
       <c r="C3">
-        <v>0.04415219721277733</v>
+        <v>0.0340817070311055</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -869,10 +1429,10 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>146.4921367429997</v>
+        <v>123.9696432960045</v>
       </c>
       <c r="C4">
-        <v>0.04069226020638881</v>
+        <v>0.03443601202666792</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -880,10 +1440,87 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>152.7449925229994</v>
+        <v>170.3926377629978</v>
       </c>
       <c r="C5">
-        <v>0.04242916458972205</v>
+        <v>0.04733128826749938</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>146.2376779089973</v>
+      </c>
+      <c r="C6">
+        <v>0.04062157719694369</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>148.7630150339974</v>
+      </c>
+      <c r="C7">
+        <v>0.04132305973166593</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>148.5343487640203</v>
+      </c>
+      <c r="C8">
+        <v>0.04125954132333896</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>131.7969799799903</v>
+      </c>
+      <c r="C9">
+        <v>0.03661027221666397</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>130.2887405339861</v>
+      </c>
+      <c r="C10">
+        <v>0.03619131681499615</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>121.8968714889779</v>
+      </c>
+      <c r="C11">
+        <v>0.03386024208027164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>144.63554956601</v>
+      </c>
+      <c r="C12">
+        <v>0.04017654154611389</v>
       </c>
     </row>
   </sheetData>
@@ -893,7 +1530,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -909,7 +1546,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>-0.7003535477870032</v>
+        <v>-0.7180226373303757</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -917,7 +1554,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>-0.06089253323748206</v>
+        <v>0.3424066203579322</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -925,7 +1562,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.766493380329111</v>
+        <v>0.8447063322470141</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -933,7 +1570,63 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.9316981584959445</v>
+        <v>0.8447063322470142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0.8447063322470141</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>0.8447063322470143</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>0.8447063322470139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>0.8447063322470142</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>0.8447063322470141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>0.8447063322470143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>0.8447063322470139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>